<commit_message>
Remove priority column from all TC tables
- README.md: 모든 테이블에서 우선순위 컬럼 제거 (ID/TC/수행테스트/기대결과 4컬럼)
- E2E_TestCases.xlsx: 우선순위 없이 재생성 (210 TC, 28 시트)
- 요약 테이블에서도 우선순위 분포 제거

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/E2E_TestCases.xlsx
+++ b/E2E_TestCases.xlsx
@@ -37,33 +37,33 @@
     <sheet name="EDGE-07. 반응형뷰포트 Edge Cases" sheetId="28" state="visible" r:id="rId28"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'TC-01. 수업 일정 관리 mainclass-mgmt'!$A$1:$E$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'TC-02. 진행자 근무 관리 mainschedule'!$A$1:$E$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'TC-03. 모니터 대시보드 monitor-dashboa'!$A$1:$E$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'TC-04. 사용자 관리 mainuser'!$A$1:$E$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'TC-05. 활동 관리 mainactivity'!$A$1:$E$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'TC-06. 메시지 관리 mainmessage'!$A$1:$E$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'TC-07. 리소스 관리 mainres'!$A$1:$E$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'TC-08. 아바타 관리 mainavatars'!$A$1:$E$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'TC-09. 활동 템플릿 mainactivity-temp'!$A$1:$E$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'TC-10. 회기 템플릿 mainlesson-templa'!$A$1:$E$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'TC-11. 커리큘럼 관리 maincurriculum'!$A$1:$E$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'TC-12. 프롬프트 변수 mainprompt-varia'!$A$1:$E$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'TC-13. 로그 mainlog'!$A$1:$E$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'TC-14. 프롬프트 테스트 mainprompt-test'!$A$1:$E$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'TC-15. 비상용 수업 main'!$A$1:$E$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'TC-16. 권한 관리 mainmember'!$A$1:$E$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'TC-17. 세션 E2E - 게스트호스트 진입 멀티탭'!$A$1:$E$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'TC-18. 세션 E2E - 활동 전환리소스AI캐릭터 멀'!$A$1:$E$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'TC-19. 세션 E2E - 호스트 컨트롤 멀티탭'!$A$1:$E$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'TC-20. 네비게이션 공통'!$A$1:$E$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'EDGE-01. 인증 Edge Cases'!$A$1:$E$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'EDGE-02. 네비게이션 Edge Cases'!$A$1:$E$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'EDGE-03. 입력 검증 Edge Cases'!$A$1:$E$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'EDGE-04. 게스트 입장 Edge Cases'!$A$1:$E$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="25" hidden="1">'EDGE-05. 세션 Edge Cases 멀티탭'!$A$1:$E$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="26" hidden="1">'EDGE-06. 페이지 안정성 Edge Cases'!$A$1:$E$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'EDGE-07. 반응형뷰포트 Edge Cases'!$A$1:$E$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'TC-01. 수업 일정 관리 mainclass-mgmt'!$A$1:$D$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'TC-02. 진행자 근무 관리 mainschedule'!$A$1:$D$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'TC-03. 모니터 대시보드 monitor-dashboa'!$A$1:$D$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'TC-04. 사용자 관리 mainuser'!$A$1:$D$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'TC-05. 활동 관리 mainactivity'!$A$1:$D$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'TC-06. 메시지 관리 mainmessage'!$A$1:$D$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'TC-07. 리소스 관리 mainres'!$A$1:$D$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'TC-08. 아바타 관리 mainavatars'!$A$1:$D$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'TC-09. 활동 템플릿 mainactivity-temp'!$A$1:$D$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'TC-10. 회기 템플릿 mainlesson-templa'!$A$1:$D$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'TC-11. 커리큘럼 관리 maincurriculum'!$A$1:$D$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'TC-12. 프롬프트 변수 mainprompt-varia'!$A$1:$D$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'TC-13. 로그 mainlog'!$A$1:$D$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'TC-14. 프롬프트 테스트 mainprompt-test'!$A$1:$D$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'TC-15. 비상용 수업 main'!$A$1:$D$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'TC-16. 권한 관리 mainmember'!$A$1:$D$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'TC-17. 세션 E2E - 게스트호스트 진입 멀티탭'!$A$1:$D$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'TC-18. 세션 E2E - 활동 전환리소스AI캐릭터 멀'!$A$1:$D$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'TC-19. 세션 E2E - 호스트 컨트롤 멀티탭'!$A$1:$D$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'TC-20. 네비게이션 공통'!$A$1:$D$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'EDGE-01. 인증 Edge Cases'!$A$1:$D$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'EDGE-02. 네비게이션 Edge Cases'!$A$1:$D$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'EDGE-03. 입력 검증 Edge Cases'!$A$1:$D$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'EDGE-04. 게스트 입장 Edge Cases'!$A$1:$D$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="25" hidden="1">'EDGE-05. 세션 Edge Cases 멀티탭'!$A$1:$D$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="26" hidden="1">'EDGE-06. 페이지 안정성 Edge Cases'!$A$1:$D$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'EDGE-07. 반응형뷰포트 Edge Cases'!$A$1:$D$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -96,7 +96,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -106,26 +106,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002B579A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEF9E7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EBF5FB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FADBD8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F3F4"/>
       </patternFill>
     </fill>
     <fill>
@@ -141,6 +121,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D5F5E3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FADBD8"/>
       </patternFill>
     </fill>
   </fills>
@@ -170,19 +155,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -196,19 +181,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1050,14 +1023,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1081,11 +1053,6 @@
           <t>기대 결과</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
-          <t>우선순위</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -1108,11 +1075,6 @@
           <t>"템플릿 목록" 제목 + 템플릿 테이블 표시</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -1135,11 +1097,6 @@
           <t>No/Template Title/Avatar/StepTitle/StepType/ActionType/ResourceType/발화유도멘트/넘어가기옵션/넘어가기조건/종속회기 컬럼 존재</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -1162,11 +1119,6 @@
           <t>1개 이상의 템플릿이 테이블에 표시</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -1189,11 +1141,6 @@
           <t>템플릿 생성 폼 표시 (필수 필드 입력 가능)</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -1216,14 +1163,9 @@
           <t>해당 템플릿의 상세 편집 화면으로 이동</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E6"/>
+  <autoFilter ref="A1:D6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1234,14 +1176,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1265,11 +1206,6 @@
           <t>기대 결과</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
-          <t>우선순위</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -1292,11 +1228,6 @@
           <t>"회기 템플릿 관리" 제목 + 회기 선택 드롭다운 + 수정/생성 버튼 표시</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -1319,11 +1250,6 @@
           <t>해당 회기에 포함된 활동 목록이 우측/하단에 로드 표시</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -1346,11 +1272,6 @@
           <t>선택된 회기의 수정 모드 진입 (활동 추가/삭제/순서변경 가능)</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -1373,14 +1294,9 @@
           <t>빈 회기 템플릿 생성 폼 표시 (이름/활동 구성 입력 가능)</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E5"/>
+  <autoFilter ref="A1:D5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1391,14 +1307,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1422,11 +1337,6 @@
           <t>기대 결과</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
-          <t>우선순위</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -1449,11 +1359,6 @@
           <t>"커리큘럼 관리" 제목 + 좌측 커리큘럼 사이드바 + 우측 상세 영역 표시</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -1476,11 +1381,6 @@
           <t>1개 이상의 커리큘럼 항목이 사이드바에 목록 형태로 표시</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -1503,11 +1403,6 @@
           <t>우측에 해당 커리큘럼의 회기 목록(회기번호/회기템플릿/활동 수) 로드</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -1530,11 +1425,6 @@
           <t>사이드바에 키워드를 포함하는 커리큘럼만 필터링 표시</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -1557,11 +1447,6 @@
           <t>커리큘럼 이름/설명 입력 폼 표시</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -1584,11 +1469,6 @@
           <t>해당 회기의 활동 구성 상세 정보 표시</t>
         </is>
       </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -1611,14 +1491,9 @@
           <t>해당 커리큘럼이 사이드바에서 제거됨</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E8"/>
+  <autoFilter ref="A1:D8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1629,14 +1504,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1660,11 +1534,6 @@
           <t>기대 결과</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
-          <t>우선순위</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -1687,11 +1556,6 @@
           <t>"프롬프트 변수 관리" 제목 + 태그 필터 칩 + 변수 카드 목록 표시</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -1714,11 +1578,6 @@
           <t>해당 태그가 포함된 변수 카드만 필터링 표시, 클릭된 태그 활성 상태</t>
         </is>
       </c>
-      <c r="E3" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -1741,11 +1600,6 @@
           <t>입력한 태그와 일치하는 변수만 필터링 표시</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -1768,11 +1622,6 @@
           <t>변수 카드 목록에 새 변수 카드 추가, 총 개수 +1</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -1795,11 +1644,6 @@
           <t>변수명/사용 템플릿 수/태그/프롬프트 내용이 카드에 표시</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -1822,14 +1666,9 @@
           <t>"N VARIABLES" 텍스트가 실제 변수 카드 수와 일치</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E7"/>
+  <autoFilter ref="A1:D7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1840,14 +1679,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1871,11 +1709,6 @@
           <t>기대 결과</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
-          <t>우선순위</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -1898,11 +1731,6 @@
           <t>"핑퐁이 세션 로그" 제목 + 사용자/회기 드롭다운 + 조회 버튼 + 로그 테이블 표시</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -1925,11 +1753,6 @@
           <t>회기 드롭다운이 활성화되고, 해당 아동의 회기 옵션이 로드</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -1952,11 +1775,6 @@
           <t>회기 번호가 선택되고, 조회 가능 상태</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -1979,11 +1797,6 @@
           <t>선택된 기간 버튼 활성, 해당 기간 범위 표시</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -2006,11 +1819,6 @@
           <t>로그 테이블의 정렬 순서가 Created At 기준으로 변경</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -2033,11 +1841,6 @@
           <t>필터 조건에 맞는 세션 로그가 테이블에 로드, 행 1개 이상 표시</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -2060,11 +1863,6 @@
           <t>Activity명/Role/Type/Message/Issue Text/Created At/진행자 개입 컬럼 존재</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -2087,14 +1885,9 @@
           <t>클립보드에 전체 로그 내용이 텍스트로 복사됨</t>
         </is>
       </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E9"/>
+  <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2105,14 +1898,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2136,11 +1928,6 @@
           <t>기대 결과</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
-          <t>우선순위</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -2163,11 +1950,6 @@
           <t>사용자/회기 드롭다운 + V1.0/V1.5 버전 토글 + Settings 버튼 + 채팅 영역 표시</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -2190,11 +1972,6 @@
           <t>회기 드롭다운 활성화, 해당 아동의 회기 옵션 로드</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -2217,11 +1994,6 @@
           <t>좌측에 해당 회기의 활동 목록(StepTitle) 표시, 선택 가능</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -2244,11 +2016,6 @@
           <t>V1.5 버튼 활성 상태, 프롬프트 버전이 1.5로 전환</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -2271,11 +2038,6 @@
           <t>설정 패널 열림 (파라미터/옵션 조정 가능), 재클릭 시 닫힘</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -2298,11 +2060,6 @@
           <t>사용자 메시지가 채팅 영역에 표시, 잠시 후 AI 응답 메시지가 추가됨</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -2325,14 +2082,9 @@
           <t>채팅 컨텍스트가 선택된 활동으로 전환, 해당 활동 프롬프트 기반 대화 가능</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E8"/>
+  <autoFilter ref="A1:D8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2343,14 +2095,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2374,11 +2125,6 @@
           <t>기대 결과</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
-          <t>우선순위</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -2401,11 +2147,6 @@
           <t>아동/회기/디바이스 3개 드롭다운 + "수업 시작" 버튼 + "현재 생성된 방 목록" 영역 표시</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -2428,11 +2169,6 @@
           <t>회기 드롭다운이 활성화, 해당 아동의 회기 번호 옵션 로드</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -2455,11 +2191,6 @@
           <t>사용 가능한 디바이스 옵션 목록 표시, 선택 가능</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -2482,11 +2213,6 @@
           <t>방이 생성되고, "현재 생성된 방 목록"에 새 방 항목 추가</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -2509,11 +2235,6 @@
           <t>생성된 방이 목록에 표시 (아동이름/회기/상태)</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -2536,14 +2257,9 @@
           <t>"생성된 방이 없습니다" 텍스트 표시</t>
         </is>
       </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E7"/>
+  <autoFilter ref="A1:D7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2554,14 +2270,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2585,11 +2300,6 @@
           <t>기대 결과</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
-          <t>우선순위</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -2612,11 +2322,6 @@
           <t>"권한 관리" 제목 + 멤버 테이블 표시</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -2639,11 +2344,6 @@
           <t>이름/역할/전화번호/Slack ID 컬럼 존재</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -2666,11 +2366,6 @@
           <t>"개발자"/"관리자"/"진행자" 등 역할이 구분되어 표시</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -2693,11 +2388,6 @@
           <t>멤버 테이블에 새 멤버 행 추가됨</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -2720,14 +2410,9 @@
           <t>1명 이상의 멤버가 테이블에 표시</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E6"/>
+  <autoFilter ref="A1:D6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2738,14 +2423,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2769,11 +2453,6 @@
           <t>기대 결과</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
-          <t>우선순위</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -2796,11 +2475,6 @@
           <t>클립보드에 `/client-guest?mode=test` URL이 복사됨</t>
         </is>
       </c>
-      <c r="E2" s="13" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -2823,11 +2497,6 @@
           <t>이름/전화번호/수업인덱스 3개 입력 필드 + "입장하기" 버튼(비활성) 표시</t>
         </is>
       </c>
-      <c r="E3" s="13" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -2850,11 +2519,6 @@
           <t>3개 필드 모두 값 입력됨, "입장하기" 버튼이 활성(enabled) 상태로 변경</t>
         </is>
       </c>
-      <c r="E4" s="13" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -2877,11 +2541,6 @@
           <t>"이전에 진행한 수업이 있어요" 다이얼로그 표시 (처음부터/이어하기 옵션) 또는 바로 리소스 로딩 시작</t>
         </is>
       </c>
-      <c r="E5" s="13" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -2904,11 +2563,6 @@
           <t>"친구가 만날 준비를 하고 있어요!" 텍스트 + 진행바(0/N → N/N) 표시 후 로딩 완료</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -2931,11 +2585,6 @@
           <t>게스트 세션 화면 진입: 배경 + AI 아바타 영역 + 좌하단 카메라 표시</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -2958,11 +2607,6 @@
           <t>`&lt;video&gt;` 요소가 visible 상태, 카메라 피드(fake device) 스트림 표시</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -2985,11 +2629,6 @@
           <t>"테스트 세션 &gt; 1:1 모니터링"에 "해리_17회기" 텍스트 + 초록 접속 표시등</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -3012,11 +2651,6 @@
           <t>호스트 모니터링 페이지 이동 (URL: `/monitor-dashboard/미지정/{roomId}?mode=test&amp;type=oneOnOne`)</t>
         </is>
       </c>
-      <c r="E10" s="13" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -3039,11 +2673,6 @@
           <t>다이얼로그 닫힘, 호스트 모니터링 UI 전체 활성화</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -3066,11 +2695,6 @@
           <t>"ACTIVITY/STEP" 헤더 + 활동 목록(공통_공통_체크인, 스몰톡, 공통_공통_송사탕 등) 표시</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
@@ -3093,11 +2717,6 @@
           <t>"Next →" 버튼 표시, 클릭 가능 상태</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -3120,11 +2739,6 @@
           <t>게스트 웹캠 스트림이 영상으로 표시</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
@@ -3147,11 +2761,6 @@
           <t>AI 아바타 캐릭터가 영상으로 표시</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -3174,11 +2783,6 @@
           <t>메시지 입력 필드(placeholder: "메시지 입력...(포커스: ⌘+M)") + "전송" 버튼 표시</t>
         </is>
       </c>
-      <c r="E16" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
@@ -3201,14 +2805,9 @@
           <t>AI 발화 메시지(예: "안녕? 만나서 반가워!")가 타임스탬프와 함께 표시</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E17"/>
+  <autoFilter ref="A1:D17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3219,14 +2818,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3250,11 +2848,6 @@
           <t>기대 결과</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
-          <t>우선순위</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -3277,11 +2870,6 @@
           <t>좌측 Activity Step에서 다음 활동이 하이라이트, AI Screen 콘텐츠 변경</t>
         </is>
       </c>
-      <c r="E2" s="13" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -3304,11 +2892,6 @@
           <t>좌측 활동 목록에서 현재 활동이 파란 테두리/하이라이트로 표시, 이전 활동은 비활성</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -3331,11 +2914,6 @@
           <t>게스트 화면의 AI 아바타/배경/콘텐츠가 새 활동에 맞게 동기화 변경</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -3358,11 +2936,6 @@
           <t>호스트 AI Screen에 이미지가 표시, `&lt;img&gt;` 요소 visible</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -3385,11 +2958,6 @@
           <t>게스트 화면에 이미지 표시 (화면 분할: 이미지 + AI 아바타)</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -3412,11 +2980,6 @@
           <t>호스트 AI Screen에 비디오 재생, 진행바(시크바) 표시</t>
         </is>
       </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -3439,11 +3002,6 @@
           <t>게스트 화면에 전체화면 비디오 재생</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -3466,11 +3024,6 @@
           <t>호스트 AI Screen에 이전과 다른 AI 캐릭터가 렌더링 (예: 지우→나은)</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -3493,14 +3046,9 @@
           <t>게스트 화면의 AI 캐릭터가 새 캐릭터로 변경되어 표시</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E10"/>
+  <autoFilter ref="A1:D10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3511,14 +3059,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3542,11 +3089,6 @@
           <t>기대 결과</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
-          <t>우선순위</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -3569,11 +3111,6 @@
           <t>"수업 일정 관리" 제목 표시, 오늘수업/전체수업/중단관리 3개 탭 노출</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -3596,11 +3133,6 @@
           <t>오늘 날짜 기준 수업 목록 테이블 표시 (시간/아동/담당자/회기/커리큘럼/진행자/상태/입장 컬럼)</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -3623,11 +3155,6 @@
           <t>전체 수업 목록이 로드되고, "전체 수업" 탭이 활성 상태로 변경</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -3650,11 +3177,6 @@
           <t>중단 수업 관리 화면 표시, "중단 관리" 탭 활성</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -3677,11 +3199,6 @@
           <t>이름에 "테스트"가 포함된 아동만 필터링되어 테이블에 표시</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -3704,11 +3221,6 @@
           <t>선택한 진행자의 수업만 테이블에 표시</t>
         </is>
       </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -3731,11 +3243,6 @@
           <t>선택한 커리큘럼의 수업만 테이블에 표시</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -3758,11 +3265,6 @@
           <t>다음 날짜로 이동, 해당 날짜의 수업 목록 표시</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -3785,11 +3287,6 @@
           <t>오늘 날짜로 복귀, 오늘의 수업 목록 표시</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -3812,11 +3309,6 @@
           <t>수업 추가 모달 표시 (아동검색/날짜/시간/진행자/사유 입력 필드)</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -3839,11 +3331,6 @@
           <t>모달 닫힘, 수업 목록에 새 수업 항목 추가됨</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
@@ -3866,11 +3353,6 @@
           <t>모달 닫힘, 수업 목록 변경 없음</t>
         </is>
       </c>
-      <c r="E13" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -3893,11 +3375,6 @@
           <t>선택된 수업이 목록에서 제거됨</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
@@ -3920,11 +3397,6 @@
           <t>접속 우회 정책 설정 모달/패널 표시</t>
         </is>
       </c>
-      <c r="E15" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -3947,11 +3419,6 @@
           <t>해당 수업의 호스트 모니터링 페이지(`/monitor-dashboard/...`)로 이동</t>
         </is>
       </c>
-      <c r="E16" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
@@ -3974,14 +3441,9 @@
           <t>대시보드 타이머 시작, 버튼 텍스트가 경과 시간으로 변경</t>
         </is>
       </c>
-      <c r="E17" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E17"/>
+  <autoFilter ref="A1:D17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3992,14 +3454,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4023,11 +3484,6 @@
           <t>기대 결과</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
-          <t>우선순위</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -4050,11 +3506,6 @@
           <t>토글 활성, AI 대화 종료 시 자동으로 다음 활동으로 전환 시작</t>
         </is>
       </c>
-      <c r="E2" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -4077,11 +3528,6 @@
           <t>채팅 로그에 "테스트 메시지"가 진행자 메시지로 표시, 게스트 측 AI가 반응</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -4104,11 +3550,6 @@
           <t>채팅 영역이 STT(음성인식) 텍스트만 표시하는 뷰로 전환</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -4131,11 +3572,6 @@
           <t>각 토글 상태 변경 (ON↔OFF), AI의 듣기/끼어들기 동작 제어</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -4158,11 +3594,6 @@
           <t>AI 아바타의 눈 상태가 변경됨 (게스트 측에서도 동기화 확인)</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -4185,11 +3616,6 @@
           <t>클릭한 프리셋에 해당하는 메시지/명령이 즉시 실행, 채팅 로그에 반영</t>
         </is>
       </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -4212,11 +3638,6 @@
           <t>"회기 종료" 모달 표시: 완료(✅)/중단(⚠)/취소(✖) 3개 옵션</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -4239,11 +3660,6 @@
           <t>세션 정상 종료, 모니터 대시보드로 복귀, 세션 목록에서 해당 세션 제거</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -4266,11 +3682,6 @@
           <t>세션 중단 기록 저장, 모니터 대시보드로 복귀</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -4293,11 +3704,6 @@
           <t>게스트가 세션에서 강제 퇴장, 게스트 화면에 "DISCONNECTED" 표시</t>
         </is>
       </c>
-      <c r="E11" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -4320,11 +3726,6 @@
           <t>회기가 첫 번째 활동으로 초기화, 모든 진행 상태 리셋</t>
         </is>
       </c>
-      <c r="E12" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
@@ -4347,11 +3748,6 @@
           <t>이슈 로그 목록에 새 이슈 항목 추가 (타임스탬프/카테고리/내용)</t>
         </is>
       </c>
-      <c r="E13" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -4374,14 +3770,9 @@
           <t>모든 이슈 로그가 서버에 저장됨, 저장 완료 알림/피드백 표시</t>
         </is>
       </c>
-      <c r="E14" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E14"/>
+  <autoFilter ref="A1:D14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4392,14 +3783,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4423,11 +3813,6 @@
           <t>기대 결과</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
-          <t>우선순위</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -4450,11 +3835,6 @@
           <t>16개 탭(수업일정/진행자근무관리/모니터대시보드/사용자/활동/메시지/리소스/아바타/활동템플릿/회기템플릿/커리큘럼/프롬프트변수/로그/테스트/(비상용)수업/권한관리) 모두 표시</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -4477,11 +3857,6 @@
           <t>"관리자 해리" 텍스트 표시</t>
         </is>
       </c>
-      <c r="E3" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -4504,11 +3879,6 @@
           <t>URL이 `/main/class-mgmt`로 변경, "수업 일정 관리" 페이지 로드</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -4531,11 +3901,6 @@
           <t>URL이 `/main/schedule`로 변경, "진행자 일정 관리" 페이지 로드</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -4558,11 +3923,6 @@
           <t>URL이 `/monitor-dashboard`로 변경, "모니터 대시보드" 페이지 로드</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -4585,11 +3945,6 @@
           <t>URL이 `/main/user`로 변경, "사용자 관리" 페이지 로드</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -4612,11 +3967,6 @@
           <t>URL이 `/main/activity`로 변경, "활동 목록" 페이지 로드</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -4639,11 +3989,6 @@
           <t>URL이 `/main/message`로 변경, 메시지 관리 페이지 로드</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -4666,11 +4011,6 @@
           <t>URL이 `/main/res`로 변경, 리소스 관리 페이지 로드</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -4693,11 +4033,6 @@
           <t>URL이 `/main/avatars`로 변경, "아바타 관리" 페이지 로드</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -4720,11 +4055,6 @@
           <t>URL이 `/main/activity-template`로 변경, "템플릿 목록" 페이지 로드</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
@@ -4747,11 +4077,6 @@
           <t>URL이 `/main/lesson-template`로 변경, "회기 템플릿 관리" 페이지 로드</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -4774,11 +4099,6 @@
           <t>URL이 `/main/curriculum`로 변경, "커리큘럼 관리" 페이지 로드</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
@@ -4801,11 +4121,6 @@
           <t>URL이 `/main/prompt-variable`로 변경, "프롬프트 변수 관리" 페이지 로드</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -4828,11 +4143,6 @@
           <t>URL이 `/main/log`로 변경, "핑퐁이 세션 로그" 페이지 로드</t>
         </is>
       </c>
-      <c r="E16" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
@@ -4855,11 +4165,6 @@
           <t>URL이 `/main/prompt-test`로 변경, 프롬프트 테스트 페이지 로드</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
@@ -4882,11 +4187,6 @@
           <t>URL이 `/main`으로 변경, 비상용 수업 페이지 로드</t>
         </is>
       </c>
-      <c r="E18" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
@@ -4909,14 +4209,9 @@
           <t>URL이 `/main/member`로 변경, "권한 관리" 페이지 로드</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E19"/>
+  <autoFilter ref="A1:D19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4927,40 +4222,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>테스트 케이스</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>수행 테스트</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>기대 결과</t>
-        </is>
-      </c>
-      <c r="E1" s="15" t="inlineStr">
-        <is>
-          <t>우선순위</t>
         </is>
       </c>
     </row>
@@ -4985,11 +4274,6 @@
           <t>로그인 리다이렉트 또는 빈 페이지 표시 (크래시 없음)</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -5012,11 +4296,6 @@
           <t>로그인 리다이렉트 또는 빈 페이지 표시 (크래시 없음)</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -5039,11 +4318,6 @@
           <t>로그인 실패, 로그인 페이지에 머무름 (에러 메시지 또는 재입력 유도)</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -5066,11 +4340,6 @@
           <t>로그인 실패, 로그인 페이지에 머무름</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -5093,14 +4362,9 @@
           <t>로그인 실패, 로그인 페이지에 머무름</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E6"/>
+  <autoFilter ref="A1:D6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5111,40 +4375,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>테스트 케이스</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>수행 테스트</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>기대 결과</t>
-        </is>
-      </c>
-      <c r="E1" s="15" t="inlineStr">
-        <is>
-          <t>우선순위</t>
         </is>
       </c>
     </row>
@@ -5169,11 +4427,6 @@
           <t>404 페이지 표시 또는 메인으로 리다이렉트 (크래시 없음)</t>
         </is>
       </c>
-      <c r="E2" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -5196,11 +4449,6 @@
           <t>로그인 상태 유지, "수업 일정 관리" 페이지 정상 표시</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -5223,11 +4471,6 @@
           <t>뒤로가기 시 수업 일정, 앞으로가기 시 사용자 페이지로 정확히 복원</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -5250,11 +4493,6 @@
           <t>마지막 클릭한 아바타 페이지(`/main/avatars`)에 정상 도달</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -5277,14 +4515,9 @@
           <t>크래시 없이 "수업 일정 관리" 정상 표시</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E6"/>
+  <autoFilter ref="A1:D6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5295,40 +4528,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>테스트 케이스</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>수행 테스트</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>기대 결과</t>
-        </is>
-      </c>
-      <c r="E1" s="15" t="inlineStr">
-        <is>
-          <t>우선순위</t>
         </is>
       </c>
     </row>
@@ -5353,11 +4580,6 @@
           <t>스크립트 실행되지 않음, "수업 일정 관리" 정상 표시</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -5380,11 +4602,6 @@
           <t>페이지 크래시 없이 검색 결과(없음) 또는 정상 표시</t>
         </is>
       </c>
-      <c r="E3" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -5407,11 +4624,6 @@
           <t>전체 결과 표시 또는 정상 동작</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -5434,11 +4646,6 @@
           <t>검색 결과 0건, 빈 테이블 또는 "결과 없음" 표시</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -5461,11 +4668,6 @@
           <t>서버 에러 없이 "리소스" 페이지 정상 표시</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -5488,14 +4690,9 @@
           <t>크래시 없이 필터링 동작 (결과 있음/없음 무관)</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E7"/>
+  <autoFilter ref="A1:D7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5506,40 +4703,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>테스트 케이스</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>수행 테스트</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>기대 결과</t>
-        </is>
-      </c>
-      <c r="E1" s="15" t="inlineStr">
-        <is>
-          <t>우선순위</t>
         </is>
       </c>
     </row>
@@ -5564,11 +4755,6 @@
           <t>"입장하기" 버튼 `disabled` 상태</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -5591,11 +4777,6 @@
           <t>"입장하기" 버튼 상태 확인 (비활성화 또는 서버 검증)</t>
         </is>
       </c>
-      <c r="E3" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -5618,11 +4799,6 @@
           <t>입장 실패 또는 에러 처리 (세션 화면 미진입)</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -5645,11 +4821,6 @@
           <t>숫자만 허용하거나, 입력되더라도 크래시 없음</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -5672,11 +4843,6 @@
           <t>에러 처리 또는 비활성화 (크래시 없음)</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -5699,14 +4865,9 @@
           <t>에러 처리 또는 정수 변환 (크래시 없음)</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E7"/>
+  <autoFilter ref="A1:D7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5717,40 +4878,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>테스트 케이스</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>수행 테스트</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>기대 결과</t>
-        </is>
-      </c>
-      <c r="E1" s="15" t="inlineStr">
-        <is>
-          <t>우선순위</t>
         </is>
       </c>
     </row>
@@ -5775,11 +4930,6 @@
           <t>세션 유지 또는 재연결 시도 (페이지 크래시 없음)</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -5802,11 +4952,6 @@
           <t>모달 정상 닫힘, 세션 계속 진행</t>
         </is>
       </c>
-      <c r="E3" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -5829,11 +4974,6 @@
           <t>완료/중단/취소 3개 옵션 표시, 취소 시 다이얼로그 닫히고 세션 유지</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -5856,14 +4996,9 @@
           <t>비디오 재표시 또는 재진입 화면 (크래시 없음)</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E5"/>
+  <autoFilter ref="A1:D5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5874,40 +5009,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>테스트 케이스</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>수행 테스트</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>기대 결과</t>
-        </is>
-      </c>
-      <c r="E1" s="15" t="inlineStr">
-        <is>
-          <t>우선순위</t>
         </is>
       </c>
     </row>
@@ -5932,11 +5061,6 @@
           <t>치명적 JavaScript 에러 5개 이하 (서드파티 제외)</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -5959,11 +5083,6 @@
           <t>500번대 서버 에러 응답 0건</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -5986,11 +5105,6 @@
           <t>크래시 없이 "수업 일정 관리" 정상 표시</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -6013,11 +5127,6 @@
           <t>크래시 없이 "활동" 페이지 정상 표시</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -6040,11 +5149,6 @@
           <t>비활성화(disabled) 또는 활성화 상태 정상 표시</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -6067,14 +5171,9 @@
           <t>크래시 없이 정상 동작 (입력 무시 또는 안내 메시지)</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E7"/>
+  <autoFilter ref="A1:D7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6085,40 +5184,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>테스트 케이스</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>수행 테스트</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>기대 결과</t>
-        </is>
-      </c>
-      <c r="E1" s="15" t="inlineStr">
-        <is>
-          <t>우선순위</t>
         </is>
       </c>
     </row>
@@ -6143,11 +5236,6 @@
           <t>"수업 일정 관리" 제목 표시, 크래시 없음</t>
         </is>
       </c>
-      <c r="E2" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -6170,11 +5258,6 @@
           <t>"수업 일정 관리" 정상 표시, 레이아웃 깨짐 없음</t>
         </is>
       </c>
-      <c r="E3" s="14" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -6197,14 +5280,9 @@
           <t>"모니터 대시보드" 제목 + "1:1 모니터링" 카드 표시</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E4"/>
+  <autoFilter ref="A1:D4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6215,14 +5293,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6246,11 +5323,6 @@
           <t>기대 결과</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
-          <t>우선순위</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -6273,11 +5345,6 @@
           <t>"진행자 일정 관리" 제목 표시, 고정시간표관리/임시휴무관리 2개 탭 노출</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -6300,11 +5367,6 @@
           <t>요일별(월~일) × 시간대(09:00~21:00) 격자 테이블 표시</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -6327,11 +5389,6 @@
           <t>해당 진행자의 시간표가 격자에 반영, 가능/휴무 셀 색상 변경</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -6354,11 +5411,6 @@
           <t>셀 상태가 가능↔휴무로 토글, 색상 변경</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -6381,11 +5433,6 @@
           <t>임시 휴무 등록/관리 화면 표시 (날짜/시간 선택 필드)</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -6408,14 +5455,9 @@
           <t>휴무 목록에 새 항목 추가, 시간표에 반영</t>
         </is>
       </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E7"/>
+  <autoFilter ref="A1:D7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6426,14 +5468,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6457,11 +5498,6 @@
           <t>기대 결과</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
-          <t>우선순위</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -6484,11 +5520,6 @@
           <t>"모니터 대시보드" 제목 + "실시간 세션 관리 및 테스트를 진행할 수 있습니다" 부제 표시</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -6511,11 +5542,6 @@
           <t>"실시간 세션 (15분 내 시작)" 헤더 아래 통합모니터링/1:1모니터링 카드 표시</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -6538,11 +5564,6 @@
           <t>접속 대기 중인 아동 목록(이름/회기/접속상태), "실시간 입장" 버튼 표시</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -6565,11 +5586,6 @@
           <t>해당 세션의 호스트 모니터링 페이지로 이동</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -6592,11 +5608,6 @@
           <t>"테스트 세션" 헤더 + "테스트 페이지 주소 복사" 버튼 + 통합/1:1 모니터링 카드</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -6619,11 +5630,6 @@
           <t>클립보드에 `{BASE_URL}/client-guest?mode=test` URL이 복사됨</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -6646,11 +5652,6 @@
           <t>"테스트 세션 &gt; 1:1 모니터링"에 "{이름}_{인덱스}회기" 항목이 초록 점과 함께 표시</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -6673,14 +5674,9 @@
           <t>"오늘의 예정 수업" 영역에 오늘 예정된 수업 카드(이름/커리큘럼/회기/시간) 목록 표시</t>
         </is>
       </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E9"/>
+  <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6691,14 +5687,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6722,11 +5717,6 @@
           <t>기대 결과</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
-          <t>우선순위</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -6749,11 +5739,6 @@
           <t>"사용자 관리" 제목 + 사용자 테이블 표시</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -6776,11 +5761,6 @@
           <t>아동이름/성별/생일/전화번호/비밀번호/커리큘럼/메인아바타/보조아바타/채널톡링크/이용권/작업 컬럼 존재</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -6803,11 +5783,6 @@
           <t>`tbody tr`이 1개 이상, 각 행에 사용자 데이터 표시</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -6830,11 +5805,6 @@
           <t>해당 이름을 포함하는 사용자만 테이블에 필터링 표시</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -6857,11 +5827,6 @@
           <t>사용자 목록 테이블에 새 사용자 행이 추가됨</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -6884,11 +5849,6 @@
           <t>해당 사용자 정보가 변경된 값으로 업데이트됨</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -6911,11 +5871,6 @@
           <t>해당 사용자 행이 테이블에서 제거됨</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -6938,11 +5893,6 @@
           <t>이용권 상세 관리 화면/모달 표시 (이용권 종류/기간/상태)</t>
         </is>
       </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -6965,14 +5915,9 @@
           <t>클립보드에 해당 사용자의 채널톡 URL이 복사됨</t>
         </is>
       </c>
-      <c r="E10" s="14" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E10"/>
+  <autoFilter ref="A1:D10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6983,14 +5928,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7014,11 +5958,6 @@
           <t>기대 결과</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
-          <t>우선순위</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -7041,11 +5980,6 @@
           <t>"활동 목록" 제목, 사용자/회기 드롭다운, 새회기생성/회기수정/새활동생성 버튼 3개 표시</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -7068,11 +6002,6 @@
           <t>회기 드롭다운이 활성화되고, 해당 아동의 회기 옵션이 로드</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -7095,11 +6024,6 @@
           <t>해당 회기의 활동 목록이 테이블에 표시</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -7122,11 +6046,6 @@
           <t>ID/Title/Avatar/StepTitle/StepType/ActionType/ResourceType/발화유도멘트/넘어가기옵션/넘어가기조건 컬럼 존재</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -7149,11 +6068,6 @@
           <t>회기 생성 폼/모달 표시 (회기 번호, 템플릿 선택 등)</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -7176,11 +6090,6 @@
           <t>선택된 회기의 수정 폼 표시 (활동 구성 변경 가능)</t>
         </is>
       </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -7203,11 +6112,6 @@
           <t>활동 생성 폼 표시 (Title/StepType/ActionType 등 입력 가능)</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -7230,11 +6134,6 @@
           <t>해당 활동의 상세 편집 화면 표시 (모든 필드 편집 가능)</t>
         </is>
       </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -7257,14 +6156,9 @@
           <t>활동 순서가 변경되고, 변경된 순서가 테이블에 반영</t>
         </is>
       </c>
-      <c r="E10" s="14" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E10"/>
+  <autoFilter ref="A1:D10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7275,14 +6169,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7306,11 +6199,6 @@
           <t>기대 결과</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
-          <t>우선순위</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -7333,11 +6221,6 @@
           <t>메시지 입력창 + "생성" 버튼 + 메시지 목록 테이블 표시</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -7360,11 +6243,6 @@
           <t>메시지 목록 테이블에 새 메시지 행 추가 (메시지/생성일)</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -7387,11 +6265,6 @@
           <t>기존 메시지가 메시지/생성일 컬럼과 함께 표시</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -7414,11 +6287,6 @@
           <t>메시지 순서가 변경되고 저장됨</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -7441,11 +6309,6 @@
           <t>해당 메시지가 목록에서 제거됨</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -7468,11 +6331,6 @@
           <t>"진행자 알림 메시지" 헤더 + 알림 규칙 목록 표시</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -7495,11 +6353,6 @@
           <t>조건(변수/비교연산자/값) + 알림 메시지 입력 폼 표시</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -7522,11 +6375,6 @@
           <t>토글 상태 변경 (ON↔OFF), 비활성 시 규칙 미적용</t>
         </is>
       </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -7549,11 +6397,6 @@
           <t>"알림톡 메시지 템플릿" 헤더 + 템플릿 목록 표시</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -7576,14 +6419,9 @@
           <t>템플릿 이름/내용 입력 폼 표시</t>
         </is>
       </c>
-      <c r="E11" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E11"/>
+  <autoFilter ref="A1:D11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7594,14 +6432,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7625,11 +6462,6 @@
           <t>기대 결과</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
-          <t>우선순위</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -7652,11 +6484,6 @@
           <t>"리소스 업로드" 영역 + "리소스 목록" 영역 표시</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -7679,11 +6506,6 @@
           <t>"클릭하거나 파일을 드래그하여 업로드" 텍스트 표시, 드래그 영역 활성</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -7706,11 +6528,6 @@
           <t>파일명에 키워드가 포함된 리소스만 테이블에 필터링 표시</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -7733,11 +6550,6 @@
           <t>체크박스/미리보기/이름/타입/크기/업데이트 컬럼 존재</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -7760,11 +6572,6 @@
           <t>"총 N개" 텍스트가 실제 리소스 수와 일치</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -7787,11 +6594,6 @@
           <t>체크박스 선택 상태로 변경, 선택된 항목 수 표시</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -7814,11 +6616,6 @@
           <t>업로드 진행 표시 → 완료 후 리소스 목록에 새 파일 추가, 총 개수 +1</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -7841,14 +6638,9 @@
           <t>선택된 리소스가 목록에서 제거, 총 개수 -1</t>
         </is>
       </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E9"/>
+  <autoFilter ref="A1:D9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7859,14 +6651,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7890,11 +6681,6 @@
           <t>기대 결과</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
-        <is>
-          <t>우선순위</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -7917,11 +6703,6 @@
           <t>"아바타 관리" 제목 + 아바타 테이블 표시</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -7944,11 +6725,6 @@
           <t>ID/이름/음성/업데이트 컬럼 존재</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -7971,11 +6747,6 @@
           <t>1개 이상의 아바타가 테이블에 표시 (ID, 이름, 음성 정보 포함)</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -7998,11 +6769,6 @@
           <t>아바타 생성 폼 표시 (이름/음성/이미지 입력 가능)</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -8025,14 +6791,9 @@
           <t>해당 아바타의 상세 편집 화면 표시</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E6"/>
+  <autoFilter ref="A1:D6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>